<commit_message>
docs: harden backtest-ksj methodology disclosures
</commit_message>
<xml_diff>
--- a/backtest-ksj/results/backtest_summary.xlsx
+++ b/backtest-ksj/results/backtest_summary.xlsx
@@ -5025,7 +5025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5047,7 +5047,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Point-in-Time 시가총액 상위 300 (KOSPI+KOSDAQ, 분기 시총 ffill, 생존편향 없음)</t>
+          <t>Point-in-Time 시가총액 상위 300 (KOSPI+KOSDAQ, 분기 시총 ffill; 현재 생존자 전용 리스트는 아님. 단, 원천 캐시 커버리지 한계 존재)</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>KODEX 200 (벤치마크)</t>
+          <t>KODEX 200 (벤치마크), 가격수익률 기준(분배금·세금 미반영)</t>
         </is>
       </c>
     </row>
@@ -5316,6 +5316,18 @@
       <c r="B28" s="9" t="inlineStr">
         <is>
           <t>리밸런싱 시점 중 n_hold==0(무투자, 현금 100%)인 비율. 위험회피 발동 또는 종목선정 실패 시 발생.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>방법론 주의</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>유니버스는 현재 생존자 전용 리스트가 아니지만 상장폐지 전체 커버리지는 원천 data/cache 범위에 의존. KODEX200 벤치마크는 분배금 재투자 총수익률이 아닌 가격수익률 기준.</t>
         </is>
       </c>
     </row>

</xml_diff>